<commit_message>
Fix Datapath and Control Signal
</commit_message>
<xml_diff>
--- a/design/graph/miniRV-全44条指令-数据通路与控制信号.xlsx
+++ b/design/graph/miniRV-全44条指令-数据通路与控制信号.xlsx
@@ -120,7 +120,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -137,6 +137,11 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -543,20 +548,20 @@
           <t>取指单元</t>
         </is>
       </c>
-      <c r="D2" s="3" t="n"/>
-      <c r="E2" s="3" t="n"/>
-      <c r="F2" s="3" t="n"/>
+      <c r="D2" s="6" t="n"/>
+      <c r="E2" s="6" t="n"/>
+      <c r="F2" s="7" t="n"/>
       <c r="G2" s="2" t="inlineStr"/>
-      <c r="H2" s="3" t="n"/>
-      <c r="I2" s="3" t="n"/>
-      <c r="J2" s="3" t="n"/>
-      <c r="K2" s="3" t="n"/>
+      <c r="H2" s="6" t="n"/>
+      <c r="I2" s="6" t="n"/>
+      <c r="J2" s="6" t="n"/>
+      <c r="K2" s="7" t="n"/>
       <c r="L2" s="2" t="inlineStr"/>
-      <c r="M2" s="3" t="n"/>
+      <c r="M2" s="7" t="n"/>
       <c r="N2" s="2" t="inlineStr"/>
-      <c r="O2" s="3" t="n"/>
-      <c r="P2" s="3" t="n"/>
-      <c r="Q2" s="3" t="n"/>
+      <c r="O2" s="6" t="n"/>
+      <c r="P2" s="6" t="n"/>
+      <c r="Q2" s="7" t="n"/>
       <c r="R2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
@@ -576,16 +581,16 @@
           <t>NPC</t>
         </is>
       </c>
-      <c r="E3" s="3" t="n"/>
-      <c r="F3" s="3" t="n"/>
+      <c r="E3" s="6" t="n"/>
+      <c r="F3" s="7" t="n"/>
       <c r="G3" s="2" t="inlineStr">
         <is>
           <t>RF</t>
         </is>
       </c>
-      <c r="H3" s="3" t="n"/>
-      <c r="I3" s="3" t="n"/>
-      <c r="J3" s="3" t="n"/>
+      <c r="H3" s="6" t="n"/>
+      <c r="I3" s="6" t="n"/>
+      <c r="J3" s="7" t="n"/>
       <c r="K3" s="2" t="inlineStr">
         <is>
           <t>SEXT</t>
@@ -596,19 +601,19 @@
           <t>ALU</t>
         </is>
       </c>
-      <c r="M3" s="3" t="n"/>
+      <c r="M3" s="7" t="n"/>
       <c r="N3" s="2" t="inlineStr">
         <is>
           <t>MREQ</t>
         </is>
       </c>
-      <c r="O3" s="3" t="n"/>
+      <c r="O3" s="7" t="n"/>
       <c r="P3" s="2" t="inlineStr">
         <is>
           <t>MEXT</t>
         </is>
       </c>
-      <c r="Q3" s="3" t="n"/>
+      <c r="Q3" s="7" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1904,7 +1909,7 @@
       </c>
       <c r="K19" s="3" t="inlineStr">
         <is>
-          <t>IN.inst[31:20]</t>
+          <t>IN.inst[31:7]</t>
         </is>
       </c>
       <c r="L19" s="3" t="inlineStr">
@@ -1987,7 +1992,7 @@
       </c>
       <c r="K20" s="3" t="inlineStr">
         <is>
-          <t>IN.inst[31:20]</t>
+          <t>IN.inst[31:7]</t>
         </is>
       </c>
       <c r="L20" s="3" t="inlineStr">
@@ -2070,7 +2075,7 @@
       </c>
       <c r="K21" s="3" t="inlineStr">
         <is>
-          <t>IN.inst[31:20]</t>
+          <t>IN.inst[31:7]</t>
         </is>
       </c>
       <c r="L21" s="3" t="inlineStr">
@@ -4150,7 +4155,7 @@
       </c>
       <c r="L46" s="3" t="inlineStr">
         <is>
-          <t>PC</t>
+          <t>PC.pc</t>
         </is>
       </c>
       <c r="M46" s="3" t="inlineStr">
@@ -4281,7 +4286,7 @@
       </c>
       <c r="E48" s="3" t="inlineStr">
         <is>
-          <t>SEXT.ext</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F48" s="3" t="inlineStr">
@@ -4403,7 +4408,7 @@
       <c r="L49" s="3" t="inlineStr">
         <is>
           <t>RF.rD1
-PC</t>
+PC.pc</t>
         </is>
       </c>
       <c r="M49" s="3" t="inlineStr">
@@ -4450,8 +4455,8 @@
           <t>npc_op</t>
         </is>
       </c>
-      <c r="E50" s="3" t="n"/>
-      <c r="F50" s="3" t="n"/>
+      <c r="E50" s="6" t="n"/>
+      <c r="F50" s="7" t="n"/>
       <c r="G50" s="2" t="inlineStr">
         <is>
           <t>-</t>
@@ -4482,7 +4487,7 @@
           <t>alu_op</t>
         </is>
       </c>
-      <c r="M50" s="3" t="n"/>
+      <c r="M50" s="7" t="n"/>
       <c r="N50" s="4" t="inlineStr">
         <is>
           <t>ram_rop</t>
@@ -4498,7 +4503,7 @@
           <t>ram_rop</t>
         </is>
       </c>
-      <c r="Q50" s="3" t="n"/>
+      <c r="Q50" s="7" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -4517,8 +4522,8 @@
           <t>-</t>
         </is>
       </c>
-      <c r="E51" s="3" t="n"/>
-      <c r="F51" s="3" t="n"/>
+      <c r="E51" s="6" t="n"/>
+      <c r="F51" s="7" t="n"/>
       <c r="G51" s="2" t="inlineStr">
         <is>
           <t>-</t>
@@ -4569,7 +4574,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="Q51" s="3" t="n"/>
+      <c r="Q51" s="7" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -4588,8 +4593,8 @@
           <t>-</t>
         </is>
       </c>
-      <c r="E52" s="3" t="n"/>
-      <c r="F52" s="3" t="n"/>
+      <c r="E52" s="6" t="n"/>
+      <c r="F52" s="7" t="n"/>
       <c r="G52" s="2" t="inlineStr">
         <is>
           <t>-</t>
@@ -4621,7 +4626,7 @@
 is_div</t>
         </is>
       </c>
-      <c r="M52" s="3" t="n"/>
+      <c r="M52" s="7" t="n"/>
       <c r="N52" s="2" t="inlineStr">
         <is>
           <t>-</t>
@@ -4637,7 +4642,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="Q52" s="3" t="n"/>
+      <c r="Q52" s="7" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="18">
@@ -4724,13 +4729,13 @@
           <t>控制信号</t>
         </is>
       </c>
-      <c r="F2" s="3" t="n"/>
-      <c r="G2" s="3" t="n"/>
-      <c r="H2" s="3" t="n"/>
-      <c r="I2" s="3" t="n"/>
-      <c r="J2" s="3" t="n"/>
-      <c r="K2" s="3" t="n"/>
-      <c r="L2" s="3" t="n"/>
+      <c r="F2" s="6" t="n"/>
+      <c r="G2" s="6" t="n"/>
+      <c r="H2" s="6" t="n"/>
+      <c r="I2" s="6" t="n"/>
+      <c r="J2" s="6" t="n"/>
+      <c r="K2" s="6" t="n"/>
+      <c r="L2" s="7" t="n"/>
       <c r="M2" s="2" t="inlineStr"/>
       <c r="N2" s="2" t="inlineStr"/>
       <c r="O2" s="2" t="inlineStr"/>
@@ -4821,7 +4826,7 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>PC4</t>
+          <t>NPC_PC4</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
@@ -4836,7 +4841,7 @@
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>I_TYPE</t>
+          <t>EXT_I</t>
         </is>
       </c>
       <c r="I4" s="3" t="inlineStr">
@@ -4846,22 +4851,22 @@
       </c>
       <c r="J4" s="3" t="inlineStr">
         <is>
-          <t>SEL_EXT</t>
+          <t>ALU_B_EXT</t>
         </is>
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>RAM_EXT_N</t>
         </is>
       </c>
       <c r="L4" s="3" t="inlineStr">
         <is>
-          <t>SEL_RS1</t>
+          <t>ALU_A_RS1</t>
         </is>
       </c>
       <c r="M4" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>RAM_WE_N</t>
         </is>
       </c>
       <c r="N4" s="3" t="inlineStr">
@@ -4899,7 +4904,7 @@
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>PC4</t>
+          <t>NPC_PC4</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
@@ -4914,7 +4919,7 @@
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>I_TYPE</t>
+          <t>EXT_I</t>
         </is>
       </c>
       <c r="I5" s="3" t="inlineStr">
@@ -4924,22 +4929,22 @@
       </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
-          <t>SEL_EXT</t>
+          <t>ALU_B_EXT</t>
         </is>
       </c>
       <c r="K5" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>RAM_EXT_N</t>
         </is>
       </c>
       <c r="L5" s="3" t="inlineStr">
         <is>
-          <t>SEL_RS1</t>
+          <t>ALU_A_RS1</t>
         </is>
       </c>
       <c r="M5" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>RAM_WE_N</t>
         </is>
       </c>
       <c r="N5" s="3" t="inlineStr">
@@ -4977,7 +4982,7 @@
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>PC4</t>
+          <t>NPC_PC4</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
@@ -4992,7 +4997,7 @@
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>I_TYPE</t>
+          <t>EXT_I</t>
         </is>
       </c>
       <c r="I6" s="3" t="inlineStr">
@@ -5002,22 +5007,22 @@
       </c>
       <c r="J6" s="3" t="inlineStr">
         <is>
-          <t>SEL_EXT</t>
+          <t>ALU_B_EXT</t>
         </is>
       </c>
       <c r="K6" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>RAM_EXT_N</t>
         </is>
       </c>
       <c r="L6" s="3" t="inlineStr">
         <is>
-          <t>SEL_RS1</t>
+          <t>ALU_A_RS1</t>
         </is>
       </c>
       <c r="M6" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>RAM_WE_N</t>
         </is>
       </c>
       <c r="N6" s="3" t="inlineStr">
@@ -5055,7 +5060,7 @@
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>PC4</t>
+          <t>NPC_PC4</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
@@ -5070,7 +5075,7 @@
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>I_TYPE</t>
+          <t>EXT_I</t>
         </is>
       </c>
       <c r="I7" s="3" t="inlineStr">
@@ -5080,22 +5085,22 @@
       </c>
       <c r="J7" s="3" t="inlineStr">
         <is>
-          <t>SEL_EXT</t>
+          <t>ALU_B_EXT</t>
         </is>
       </c>
       <c r="K7" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>RAM_EXT_N</t>
         </is>
       </c>
       <c r="L7" s="3" t="inlineStr">
         <is>
-          <t>SEL_RS1</t>
+          <t>ALU_A_RS1</t>
         </is>
       </c>
       <c r="M7" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>RAM_WE_N</t>
         </is>
       </c>
       <c r="N7" s="3" t="inlineStr">
@@ -5133,7 +5138,7 @@
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>PC4</t>
+          <t>NPC_PC4</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
@@ -5148,7 +5153,7 @@
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
-          <t>I_TYPE</t>
+          <t>EXT_I</t>
         </is>
       </c>
       <c r="I8" s="3" t="inlineStr">
@@ -5158,22 +5163,22 @@
       </c>
       <c r="J8" s="3" t="inlineStr">
         <is>
-          <t>SEL_EXT</t>
+          <t>ALU_B_EXT</t>
         </is>
       </c>
       <c r="K8" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>RAM_EXT_N</t>
         </is>
       </c>
       <c r="L8" s="3" t="inlineStr">
         <is>
-          <t>SEL_RS1</t>
+          <t>ALU_A_RS1</t>
         </is>
       </c>
       <c r="M8" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>RAM_WE_N</t>
         </is>
       </c>
       <c r="N8" s="3" t="inlineStr">
@@ -5211,7 +5216,7 @@
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>PC4</t>
+          <t>NPC_PC4</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
@@ -5226,7 +5231,7 @@
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
-          <t>I_TYPE</t>
+          <t>EXT_I</t>
         </is>
       </c>
       <c r="I9" s="3" t="inlineStr">
@@ -5236,22 +5241,22 @@
       </c>
       <c r="J9" s="3" t="inlineStr">
         <is>
-          <t>SEL_EXT</t>
+          <t>ALU_B_EXT</t>
         </is>
       </c>
       <c r="K9" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>RAM_EXT_N</t>
         </is>
       </c>
       <c r="L9" s="3" t="inlineStr">
         <is>
-          <t>SEL_RS1</t>
+          <t>ALU_A_RS1</t>
         </is>
       </c>
       <c r="M9" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>RAM_WE_N</t>
         </is>
       </c>
       <c r="N9" s="3" t="inlineStr">
@@ -5289,7 +5294,7 @@
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>PC4</t>
+          <t>NPC_PC4</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
@@ -5304,7 +5309,7 @@
       </c>
       <c r="H10" s="3" t="inlineStr">
         <is>
-          <t>I_TYPE</t>
+          <t>EXT_I</t>
         </is>
       </c>
       <c r="I10" s="3" t="inlineStr">
@@ -5314,22 +5319,22 @@
       </c>
       <c r="J10" s="3" t="inlineStr">
         <is>
-          <t>SEL_EXT</t>
+          <t>ALU_B_EXT</t>
         </is>
       </c>
       <c r="K10" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>RAM_EXT_N</t>
         </is>
       </c>
       <c r="L10" s="3" t="inlineStr">
         <is>
-          <t>SEL_RS1</t>
+          <t>ALU_A_RS1</t>
         </is>
       </c>
       <c r="M10" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>RAM_WE_N</t>
         </is>
       </c>
       <c r="N10" s="3" t="inlineStr">
@@ -5367,7 +5372,7 @@
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>PC4</t>
+          <t>NPC_PC4</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
@@ -5382,7 +5387,7 @@
       </c>
       <c r="H11" s="3" t="inlineStr">
         <is>
-          <t>I_TYPE</t>
+          <t>EXT_I</t>
         </is>
       </c>
       <c r="I11" s="3" t="inlineStr">
@@ -5392,22 +5397,22 @@
       </c>
       <c r="J11" s="3" t="inlineStr">
         <is>
-          <t>SEL_EXT</t>
+          <t>ALU_B_EXT</t>
         </is>
       </c>
       <c r="K11" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>RAM_EXT_N</t>
         </is>
       </c>
       <c r="L11" s="3" t="inlineStr">
         <is>
-          <t>SEL_RS1</t>
+          <t>ALU_A_RS1</t>
         </is>
       </c>
       <c r="M11" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>RAM_WE_N</t>
         </is>
       </c>
       <c r="N11" s="3" t="inlineStr">
@@ -5445,7 +5450,7 @@
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>PC4</t>
+          <t>NPC_PC4</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
@@ -5460,7 +5465,7 @@
       </c>
       <c r="H12" s="3" t="inlineStr">
         <is>
-          <t>I_TYPE</t>
+          <t>EXT_I</t>
         </is>
       </c>
       <c r="I12" s="3" t="inlineStr">
@@ -5470,22 +5475,22 @@
       </c>
       <c r="J12" s="3" t="inlineStr">
         <is>
-          <t>SEL_EXT</t>
+          <t>ALU_B_EXT</t>
         </is>
       </c>
       <c r="K12" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>RAM_EXT_N</t>
         </is>
       </c>
       <c r="L12" s="3" t="inlineStr">
         <is>
-          <t>SEL_RS1</t>
+          <t>ALU_A_RS1</t>
         </is>
       </c>
       <c r="M12" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>RAM_WE_N</t>
         </is>
       </c>
       <c r="N12" s="3" t="inlineStr">
@@ -5523,7 +5528,7 @@
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>PC4</t>
+          <t>NPC_PC4</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
@@ -5538,7 +5543,7 @@
       </c>
       <c r="H13" s="3" t="inlineStr">
         <is>
-          <t>I_TYPE</t>
+          <t>EXT_I</t>
         </is>
       </c>
       <c r="I13" s="3" t="inlineStr">
@@ -5548,22 +5553,22 @@
       </c>
       <c r="J13" s="3" t="inlineStr">
         <is>
-          <t>SEL_EXT</t>
+          <t>ALU_B_EXT</t>
         </is>
       </c>
       <c r="K13" s="3" t="inlineStr">
         <is>
-          <t>WORD_EXT</t>
+          <t>RAM_EXT_W</t>
         </is>
       </c>
       <c r="L13" s="3" t="inlineStr">
         <is>
-          <t>SEL_RS1</t>
+          <t>ALU_A_RS1</t>
         </is>
       </c>
       <c r="M13" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>RAM_WE_N</t>
         </is>
       </c>
       <c r="N13" s="3" t="inlineStr">
@@ -5601,7 +5606,7 @@
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>PC4</t>
+          <t>NPC_PC4</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
@@ -5616,7 +5621,7 @@
       </c>
       <c r="H14" s="3" t="inlineStr">
         <is>
-          <t>I_TYPE</t>
+          <t>EXT_I</t>
         </is>
       </c>
       <c r="I14" s="3" t="inlineStr">
@@ -5626,22 +5631,22 @@
       </c>
       <c r="J14" s="3" t="inlineStr">
         <is>
-          <t>SEL_EXT</t>
+          <t>ALU_B_EXT</t>
         </is>
       </c>
       <c r="K14" s="3" t="inlineStr">
         <is>
-          <t>BYTE_EXT</t>
+          <t>RAM_EXT_B</t>
         </is>
       </c>
       <c r="L14" s="3" t="inlineStr">
         <is>
-          <t>SEL_RS1</t>
+          <t>ALU_A_RS1</t>
         </is>
       </c>
       <c r="M14" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>RAM_WE_N</t>
         </is>
       </c>
       <c r="N14" s="3" t="inlineStr">
@@ -5679,7 +5684,7 @@
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>PC4</t>
+          <t>NPC_PC4</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
@@ -5694,7 +5699,7 @@
       </c>
       <c r="H15" s="3" t="inlineStr">
         <is>
-          <t>I_TYPE</t>
+          <t>EXT_I</t>
         </is>
       </c>
       <c r="I15" s="3" t="inlineStr">
@@ -5704,22 +5709,22 @@
       </c>
       <c r="J15" s="3" t="inlineStr">
         <is>
-          <t>SEL_EXT</t>
+          <t>ALU_B_EXT</t>
         </is>
       </c>
       <c r="K15" s="3" t="inlineStr">
         <is>
-          <t>BYTEU_EXT</t>
+          <t>RAM_EXT_BU</t>
         </is>
       </c>
       <c r="L15" s="3" t="inlineStr">
         <is>
-          <t>SEL_RS1</t>
+          <t>ALU_A_RS1</t>
         </is>
       </c>
       <c r="M15" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>RAM_WE_N</t>
         </is>
       </c>
       <c r="N15" s="3" t="inlineStr">
@@ -5757,7 +5762,7 @@
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>PC4</t>
+          <t>NPC_PC4</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
@@ -5772,7 +5777,7 @@
       </c>
       <c r="H16" s="3" t="inlineStr">
         <is>
-          <t>I_TYPE</t>
+          <t>EXT_I</t>
         </is>
       </c>
       <c r="I16" s="3" t="inlineStr">
@@ -5782,22 +5787,22 @@
       </c>
       <c r="J16" s="3" t="inlineStr">
         <is>
-          <t>SEL_EXT</t>
+          <t>ALU_B_EXT</t>
         </is>
       </c>
       <c r="K16" s="3" t="inlineStr">
         <is>
-          <t>HALF_EXT</t>
+          <t>RAM_EXT_H</t>
         </is>
       </c>
       <c r="L16" s="3" t="inlineStr">
         <is>
-          <t>SEL_RS1</t>
+          <t>ALU_A_RS1</t>
         </is>
       </c>
       <c r="M16" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>RAM_WE_N</t>
         </is>
       </c>
       <c r="N16" s="3" t="inlineStr">
@@ -5835,7 +5840,7 @@
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>PC4</t>
+          <t>NPC_PC4</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
@@ -5850,7 +5855,7 @@
       </c>
       <c r="H17" s="3" t="inlineStr">
         <is>
-          <t>I_TYPE</t>
+          <t>EXT_I</t>
         </is>
       </c>
       <c r="I17" s="3" t="inlineStr">
@@ -5860,22 +5865,22 @@
       </c>
       <c r="J17" s="3" t="inlineStr">
         <is>
-          <t>SEL_EXT</t>
+          <t>ALU_B_EXT</t>
         </is>
       </c>
       <c r="K17" s="3" t="inlineStr">
         <is>
-          <t>HALFU_EXT</t>
+          <t>RAM_EXT_HU</t>
         </is>
       </c>
       <c r="L17" s="3" t="inlineStr">
         <is>
-          <t>SEL_RS1</t>
+          <t>ALU_A_RS1</t>
         </is>
       </c>
       <c r="M17" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>RAM_WE_N</t>
         </is>
       </c>
       <c r="N17" s="3" t="inlineStr">
@@ -5913,7 +5918,7 @@
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>PC4</t>
+          <t>NPC_PC4</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
@@ -5928,7 +5933,7 @@
       </c>
       <c r="H18" s="3" t="inlineStr">
         <is>
-          <t>I_TYPE</t>
+          <t>EXT_S</t>
         </is>
       </c>
       <c r="I18" s="3" t="inlineStr">
@@ -5938,22 +5943,22 @@
       </c>
       <c r="J18" s="3" t="inlineStr">
         <is>
-          <t>SEL_EXT</t>
+          <t>ALU_B_EXT</t>
         </is>
       </c>
       <c r="K18" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>RAM_EXT_N</t>
         </is>
       </c>
       <c r="L18" s="3" t="inlineStr">
         <is>
-          <t>SEL_RS1</t>
+          <t>ALU_A_RS1</t>
         </is>
       </c>
       <c r="M18" s="3" t="inlineStr">
         <is>
-          <t>BYTE_WE</t>
+          <t>RAM_WE_B</t>
         </is>
       </c>
       <c r="N18" s="3" t="inlineStr">
@@ -5991,7 +5996,7 @@
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>PC4</t>
+          <t>NPC_PC4</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
@@ -6006,7 +6011,7 @@
       </c>
       <c r="H19" s="3" t="inlineStr">
         <is>
-          <t>I_TYPE</t>
+          <t>EXT_S</t>
         </is>
       </c>
       <c r="I19" s="3" t="inlineStr">
@@ -6016,22 +6021,22 @@
       </c>
       <c r="J19" s="3" t="inlineStr">
         <is>
-          <t>SEL_EXT</t>
+          <t>ALU_B_EXT</t>
         </is>
       </c>
       <c r="K19" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>RAM_EXT_N</t>
         </is>
       </c>
       <c r="L19" s="3" t="inlineStr">
         <is>
-          <t>SEL_RS1</t>
+          <t>ALU_A_RS1</t>
         </is>
       </c>
       <c r="M19" s="3" t="inlineStr">
         <is>
-          <t>HALF_WE</t>
+          <t>RAM_WE_H</t>
         </is>
       </c>
       <c r="N19" s="3" t="inlineStr">
@@ -6069,7 +6074,7 @@
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>PC4</t>
+          <t>NPC_PC4</t>
         </is>
       </c>
       <c r="F20" s="3" t="inlineStr">
@@ -6084,7 +6089,7 @@
       </c>
       <c r="H20" s="3" t="inlineStr">
         <is>
-          <t>I_TYPE</t>
+          <t>EXT_S</t>
         </is>
       </c>
       <c r="I20" s="3" t="inlineStr">
@@ -6094,22 +6099,22 @@
       </c>
       <c r="J20" s="3" t="inlineStr">
         <is>
-          <t>SEL_EXT</t>
+          <t>ALU_B_EXT</t>
         </is>
       </c>
       <c r="K20" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>RAM_EXT_N</t>
         </is>
       </c>
       <c r="L20" s="3" t="inlineStr">
         <is>
-          <t>SEL_RS1</t>
+          <t>ALU_A_RS1</t>
         </is>
       </c>
       <c r="M20" s="3" t="inlineStr">
         <is>
-          <t>WORD_WE</t>
+          <t>RAM_WE_W</t>
         </is>
       </c>
       <c r="N20" s="3" t="inlineStr">
@@ -6147,7 +6152,7 @@
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>PC4</t>
+          <t>NPC_PC4</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr">
@@ -6172,22 +6177,22 @@
       </c>
       <c r="J21" s="3" t="inlineStr">
         <is>
-          <t>SEL_RS2</t>
+          <t>ALU_B_RS2</t>
         </is>
       </c>
       <c r="K21" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>RAM_EXT_N</t>
         </is>
       </c>
       <c r="L21" s="3" t="inlineStr">
         <is>
-          <t>SEL_RS1</t>
+          <t>ALU_A_RS1</t>
         </is>
       </c>
       <c r="M21" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>RAM_WE_N</t>
         </is>
       </c>
       <c r="N21" s="3" t="inlineStr">
@@ -6225,7 +6230,7 @@
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>PC4</t>
+          <t>NPC_PC4</t>
         </is>
       </c>
       <c r="F22" s="3" t="inlineStr">
@@ -6250,22 +6255,22 @@
       </c>
       <c r="J22" s="3" t="inlineStr">
         <is>
-          <t>SEL_RS2</t>
+          <t>ALU_B_RS2</t>
         </is>
       </c>
       <c r="K22" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>RAM_EXT_N</t>
         </is>
       </c>
       <c r="L22" s="3" t="inlineStr">
         <is>
-          <t>SEL_RS1</t>
+          <t>ALU_A_RS1</t>
         </is>
       </c>
       <c r="M22" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>RAM_WE_N</t>
         </is>
       </c>
       <c r="N22" s="3" t="inlineStr">
@@ -6303,7 +6308,7 @@
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>PC4</t>
+          <t>NPC_PC4</t>
         </is>
       </c>
       <c r="F23" s="3" t="inlineStr">
@@ -6328,22 +6333,22 @@
       </c>
       <c r="J23" s="3" t="inlineStr">
         <is>
-          <t>SEL_RS2</t>
+          <t>ALU_B_RS2</t>
         </is>
       </c>
       <c r="K23" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>RAM_EXT_N</t>
         </is>
       </c>
       <c r="L23" s="3" t="inlineStr">
         <is>
-          <t>SEL_RS1</t>
+          <t>ALU_A_RS1</t>
         </is>
       </c>
       <c r="M23" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>RAM_WE_N</t>
         </is>
       </c>
       <c r="N23" s="3" t="inlineStr">
@@ -6381,7 +6386,7 @@
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>PC4</t>
+          <t>NPC_PC4</t>
         </is>
       </c>
       <c r="F24" s="3" t="inlineStr">
@@ -6406,22 +6411,22 @@
       </c>
       <c r="J24" s="3" t="inlineStr">
         <is>
-          <t>SEL_RS2</t>
+          <t>ALU_B_RS2</t>
         </is>
       </c>
       <c r="K24" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>RAM_EXT_N</t>
         </is>
       </c>
       <c r="L24" s="3" t="inlineStr">
         <is>
-          <t>SEL_RS1</t>
+          <t>ALU_A_RS1</t>
         </is>
       </c>
       <c r="M24" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>RAM_WE_N</t>
         </is>
       </c>
       <c r="N24" s="3" t="inlineStr">
@@ -6459,7 +6464,7 @@
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>PC4</t>
+          <t>NPC_PC4</t>
         </is>
       </c>
       <c r="F25" s="3" t="inlineStr">
@@ -6484,22 +6489,22 @@
       </c>
       <c r="J25" s="3" t="inlineStr">
         <is>
-          <t>SEL_RS2</t>
+          <t>ALU_B_RS2</t>
         </is>
       </c>
       <c r="K25" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>RAM_EXT_N</t>
         </is>
       </c>
       <c r="L25" s="3" t="inlineStr">
         <is>
-          <t>SEL_RS1</t>
+          <t>ALU_A_RS1</t>
         </is>
       </c>
       <c r="M25" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>RAM_WE_N</t>
         </is>
       </c>
       <c r="N25" s="3" t="inlineStr">
@@ -6537,7 +6542,7 @@
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>PC4</t>
+          <t>NPC_PC4</t>
         </is>
       </c>
       <c r="F26" s="3" t="inlineStr">
@@ -6562,22 +6567,22 @@
       </c>
       <c r="J26" s="3" t="inlineStr">
         <is>
-          <t>SEL_RS2</t>
+          <t>ALU_B_RS2</t>
         </is>
       </c>
       <c r="K26" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>RAM_EXT_N</t>
         </is>
       </c>
       <c r="L26" s="3" t="inlineStr">
         <is>
-          <t>SEL_RS1</t>
+          <t>ALU_A_RS1</t>
         </is>
       </c>
       <c r="M26" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>RAM_WE_N</t>
         </is>
       </c>
       <c r="N26" s="3" t="inlineStr">
@@ -6615,7 +6620,7 @@
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>PC4</t>
+          <t>NPC_PC4</t>
         </is>
       </c>
       <c r="F27" s="3" t="inlineStr">
@@ -6640,22 +6645,22 @@
       </c>
       <c r="J27" s="3" t="inlineStr">
         <is>
-          <t>SEL_RS2</t>
+          <t>ALU_B_RS2</t>
         </is>
       </c>
       <c r="K27" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>RAM_EXT_N</t>
         </is>
       </c>
       <c r="L27" s="3" t="inlineStr">
         <is>
-          <t>SEL_RS1</t>
+          <t>ALU_A_RS1</t>
         </is>
       </c>
       <c r="M27" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>RAM_WE_N</t>
         </is>
       </c>
       <c r="N27" s="3" t="inlineStr">
@@ -6693,7 +6698,7 @@
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>PC4</t>
+          <t>NPC_PC4</t>
         </is>
       </c>
       <c r="F28" s="3" t="inlineStr">
@@ -6718,22 +6723,22 @@
       </c>
       <c r="J28" s="3" t="inlineStr">
         <is>
-          <t>SEL_RS2</t>
+          <t>ALU_B_RS2</t>
         </is>
       </c>
       <c r="K28" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>RAM_EXT_N</t>
         </is>
       </c>
       <c r="L28" s="3" t="inlineStr">
         <is>
-          <t>SEL_RS1</t>
+          <t>ALU_A_RS1</t>
         </is>
       </c>
       <c r="M28" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>RAM_WE_N</t>
         </is>
       </c>
       <c r="N28" s="3" t="inlineStr">
@@ -6771,7 +6776,7 @@
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t>PC4</t>
+          <t>NPC_PC4</t>
         </is>
       </c>
       <c r="F29" s="3" t="inlineStr">
@@ -6796,22 +6801,22 @@
       </c>
       <c r="J29" s="3" t="inlineStr">
         <is>
-          <t>SEL_RS2</t>
+          <t>ALU_B_RS2</t>
         </is>
       </c>
       <c r="K29" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>RAM_EXT_N</t>
         </is>
       </c>
       <c r="L29" s="3" t="inlineStr">
         <is>
-          <t>SEL_RS1</t>
+          <t>ALU_A_RS1</t>
         </is>
       </c>
       <c r="M29" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>RAM_WE_N</t>
         </is>
       </c>
       <c r="N29" s="3" t="inlineStr">
@@ -6849,7 +6854,7 @@
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>PC4</t>
+          <t>NPC_PC4</t>
         </is>
       </c>
       <c r="F30" s="3" t="inlineStr">
@@ -6874,22 +6879,22 @@
       </c>
       <c r="J30" s="3" t="inlineStr">
         <is>
-          <t>SEL_RS2</t>
+          <t>ALU_B_RS2</t>
         </is>
       </c>
       <c r="K30" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>RAM_EXT_N</t>
         </is>
       </c>
       <c r="L30" s="3" t="inlineStr">
         <is>
-          <t>SEL_RS1</t>
+          <t>ALU_A_RS1</t>
         </is>
       </c>
       <c r="M30" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>RAM_WE_N</t>
         </is>
       </c>
       <c r="N30" s="3" t="inlineStr">
@@ -6927,7 +6932,7 @@
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>PC4</t>
+          <t>NPC_PC4</t>
         </is>
       </c>
       <c r="F31" s="3" t="inlineStr">
@@ -6952,22 +6957,22 @@
       </c>
       <c r="J31" s="3" t="inlineStr">
         <is>
-          <t>SEL_RS2</t>
+          <t>ALU_B_RS2</t>
         </is>
       </c>
       <c r="K31" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>RAM_EXT_N</t>
         </is>
       </c>
       <c r="L31" s="3" t="inlineStr">
         <is>
-          <t>SEL_RS1</t>
+          <t>ALU_A_RS1</t>
         </is>
       </c>
       <c r="M31" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>RAM_WE_N</t>
         </is>
       </c>
       <c r="N31" s="3" t="inlineStr">
@@ -7005,7 +7010,7 @@
       </c>
       <c r="E32" s="3" t="inlineStr">
         <is>
-          <t>PC4</t>
+          <t>NPC_PC4</t>
         </is>
       </c>
       <c r="F32" s="3" t="inlineStr">
@@ -7030,22 +7035,22 @@
       </c>
       <c r="J32" s="3" t="inlineStr">
         <is>
-          <t>SEL_RS2</t>
+          <t>ALU_B_RS2</t>
         </is>
       </c>
       <c r="K32" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>RAM_EXT_N</t>
         </is>
       </c>
       <c r="L32" s="3" t="inlineStr">
         <is>
-          <t>SEL_RS1</t>
+          <t>ALU_A_RS1</t>
         </is>
       </c>
       <c r="M32" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>RAM_WE_N</t>
         </is>
       </c>
       <c r="N32" s="3" t="inlineStr">
@@ -7083,7 +7088,7 @@
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>PC4</t>
+          <t>NPC_PC4</t>
         </is>
       </c>
       <c r="F33" s="3" t="inlineStr">
@@ -7108,22 +7113,22 @@
       </c>
       <c r="J33" s="3" t="inlineStr">
         <is>
-          <t>SEL_RS2</t>
+          <t>ALU_B_RS2</t>
         </is>
       </c>
       <c r="K33" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>RAM_EXT_N</t>
         </is>
       </c>
       <c r="L33" s="3" t="inlineStr">
         <is>
-          <t>SEL_RS1</t>
+          <t>ALU_A_RS1</t>
         </is>
       </c>
       <c r="M33" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>RAM_WE_N</t>
         </is>
       </c>
       <c r="N33" s="3" t="inlineStr">
@@ -7161,7 +7166,7 @@
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>PC4</t>
+          <t>NPC_PC4</t>
         </is>
       </c>
       <c r="F34" s="3" t="inlineStr">
@@ -7186,22 +7191,22 @@
       </c>
       <c r="J34" s="3" t="inlineStr">
         <is>
-          <t>SEL_RS2</t>
+          <t>ALU_B_RS2</t>
         </is>
       </c>
       <c r="K34" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>RAM_EXT_N</t>
         </is>
       </c>
       <c r="L34" s="3" t="inlineStr">
         <is>
-          <t>SEL_RS1</t>
+          <t>ALU_A_RS1</t>
         </is>
       </c>
       <c r="M34" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>RAM_WE_N</t>
         </is>
       </c>
       <c r="N34" s="3" t="inlineStr">
@@ -7239,7 +7244,7 @@
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>PC4</t>
+          <t>NPC_PC4</t>
         </is>
       </c>
       <c r="F35" s="3" t="inlineStr">
@@ -7264,22 +7269,22 @@
       </c>
       <c r="J35" s="3" t="inlineStr">
         <is>
-          <t>SEL_RS2</t>
+          <t>ALU_B_RS2</t>
         </is>
       </c>
       <c r="K35" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>RAM_EXT_N</t>
         </is>
       </c>
       <c r="L35" s="3" t="inlineStr">
         <is>
-          <t>SEL_RS1</t>
+          <t>ALU_A_RS1</t>
         </is>
       </c>
       <c r="M35" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>RAM_WE_N</t>
         </is>
       </c>
       <c r="N35" s="3" t="inlineStr">
@@ -7317,7 +7322,7 @@
       </c>
       <c r="E36" s="3" t="inlineStr">
         <is>
-          <t>PC4</t>
+          <t>NPC_PC4</t>
         </is>
       </c>
       <c r="F36" s="3" t="inlineStr">
@@ -7342,22 +7347,22 @@
       </c>
       <c r="J36" s="3" t="inlineStr">
         <is>
-          <t>SEL_RS2</t>
+          <t>ALU_B_RS2</t>
         </is>
       </c>
       <c r="K36" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>RAM_EXT_N</t>
         </is>
       </c>
       <c r="L36" s="3" t="inlineStr">
         <is>
-          <t>SEL_RS1</t>
+          <t>ALU_A_RS1</t>
         </is>
       </c>
       <c r="M36" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>RAM_WE_N</t>
         </is>
       </c>
       <c r="N36" s="3" t="inlineStr">
@@ -7395,7 +7400,7 @@
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>PC4</t>
+          <t>NPC_PC4</t>
         </is>
       </c>
       <c r="F37" s="3" t="inlineStr">
@@ -7420,22 +7425,22 @@
       </c>
       <c r="J37" s="3" t="inlineStr">
         <is>
-          <t>SEL_RS2</t>
+          <t>ALU_B_RS2</t>
         </is>
       </c>
       <c r="K37" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>RAM_EXT_N</t>
         </is>
       </c>
       <c r="L37" s="3" t="inlineStr">
         <is>
-          <t>SEL_RS1</t>
+          <t>ALU_A_RS1</t>
         </is>
       </c>
       <c r="M37" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>RAM_WE_N</t>
         </is>
       </c>
       <c r="N37" s="3" t="inlineStr">
@@ -7473,7 +7478,7 @@
       </c>
       <c r="E38" s="3" t="inlineStr">
         <is>
-          <t>BRANCH</t>
+          <t>NPC_BRA</t>
         </is>
       </c>
       <c r="F38" s="3" t="inlineStr">
@@ -7488,7 +7493,7 @@
       </c>
       <c r="H38" s="3" t="inlineStr">
         <is>
-          <t>B_TYPE</t>
+          <t>EXT_B</t>
         </is>
       </c>
       <c r="I38" s="3" t="inlineStr">
@@ -7498,22 +7503,22 @@
       </c>
       <c r="J38" s="3" t="inlineStr">
         <is>
-          <t>SEL_RS2</t>
+          <t>ALU_B_RS2</t>
         </is>
       </c>
       <c r="K38" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>RAM_EXT_N</t>
         </is>
       </c>
       <c r="L38" s="3" t="inlineStr">
         <is>
-          <t>SEL_RS1</t>
+          <t>ALU_A_RS1</t>
         </is>
       </c>
       <c r="M38" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>RAM_WE_N</t>
         </is>
       </c>
       <c r="N38" s="3" t="inlineStr">
@@ -7551,7 +7556,7 @@
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t>BRANCH</t>
+          <t>NPC_BRA</t>
         </is>
       </c>
       <c r="F39" s="3" t="inlineStr">
@@ -7566,7 +7571,7 @@
       </c>
       <c r="H39" s="3" t="inlineStr">
         <is>
-          <t>B_TYPE</t>
+          <t>EXT_B</t>
         </is>
       </c>
       <c r="I39" s="3" t="inlineStr">
@@ -7576,22 +7581,22 @@
       </c>
       <c r="J39" s="3" t="inlineStr">
         <is>
-          <t>SEL_RS2</t>
+          <t>ALU_B_RS2</t>
         </is>
       </c>
       <c r="K39" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>RAM_EXT_N</t>
         </is>
       </c>
       <c r="L39" s="3" t="inlineStr">
         <is>
-          <t>SEL_RS1</t>
+          <t>ALU_A_RS1</t>
         </is>
       </c>
       <c r="M39" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>RAM_WE_N</t>
         </is>
       </c>
       <c r="N39" s="3" t="inlineStr">
@@ -7629,7 +7634,7 @@
       </c>
       <c r="E40" s="3" t="inlineStr">
         <is>
-          <t>BRANCH</t>
+          <t>NPC_BRA</t>
         </is>
       </c>
       <c r="F40" s="3" t="inlineStr">
@@ -7644,7 +7649,7 @@
       </c>
       <c r="H40" s="3" t="inlineStr">
         <is>
-          <t>B_TYPE</t>
+          <t>EXT_B</t>
         </is>
       </c>
       <c r="I40" s="3" t="inlineStr">
@@ -7654,22 +7659,22 @@
       </c>
       <c r="J40" s="3" t="inlineStr">
         <is>
-          <t>SEL_RS2</t>
+          <t>ALU_B_RS2</t>
         </is>
       </c>
       <c r="K40" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>RAM_EXT_N</t>
         </is>
       </c>
       <c r="L40" s="3" t="inlineStr">
         <is>
-          <t>SEL_RS1</t>
+          <t>ALU_A_RS1</t>
         </is>
       </c>
       <c r="M40" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>RAM_WE_N</t>
         </is>
       </c>
       <c r="N40" s="3" t="inlineStr">
@@ -7707,7 +7712,7 @@
       </c>
       <c r="E41" s="3" t="inlineStr">
         <is>
-          <t>BRANCH</t>
+          <t>NPC_BRA</t>
         </is>
       </c>
       <c r="F41" s="3" t="inlineStr">
@@ -7722,7 +7727,7 @@
       </c>
       <c r="H41" s="3" t="inlineStr">
         <is>
-          <t>B_TYPE</t>
+          <t>EXT_B</t>
         </is>
       </c>
       <c r="I41" s="3" t="inlineStr">
@@ -7732,22 +7737,22 @@
       </c>
       <c r="J41" s="3" t="inlineStr">
         <is>
-          <t>SEL_RS2</t>
+          <t>ALU_B_RS2</t>
         </is>
       </c>
       <c r="K41" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>RAM_EXT_N</t>
         </is>
       </c>
       <c r="L41" s="3" t="inlineStr">
         <is>
-          <t>SEL_RS1</t>
+          <t>ALU_A_RS1</t>
         </is>
       </c>
       <c r="M41" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>RAM_WE_N</t>
         </is>
       </c>
       <c r="N41" s="3" t="inlineStr">
@@ -7785,7 +7790,7 @@
       </c>
       <c r="E42" s="3" t="inlineStr">
         <is>
-          <t>BRANCH</t>
+          <t>NPC_BRA</t>
         </is>
       </c>
       <c r="F42" s="3" t="inlineStr">
@@ -7800,7 +7805,7 @@
       </c>
       <c r="H42" s="3" t="inlineStr">
         <is>
-          <t>B_TYPE</t>
+          <t>EXT_B</t>
         </is>
       </c>
       <c r="I42" s="3" t="inlineStr">
@@ -7810,22 +7815,22 @@
       </c>
       <c r="J42" s="3" t="inlineStr">
         <is>
-          <t>SEL_RS2</t>
+          <t>ALU_B_RS2</t>
         </is>
       </c>
       <c r="K42" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>RAM_EXT_N</t>
         </is>
       </c>
       <c r="L42" s="3" t="inlineStr">
         <is>
-          <t>SEL_RS1</t>
+          <t>ALU_A_RS1</t>
         </is>
       </c>
       <c r="M42" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>RAM_WE_N</t>
         </is>
       </c>
       <c r="N42" s="3" t="inlineStr">
@@ -7863,7 +7868,7 @@
       </c>
       <c r="E43" s="3" t="inlineStr">
         <is>
-          <t>BRANCH</t>
+          <t>NPC_BRA</t>
         </is>
       </c>
       <c r="F43" s="3" t="inlineStr">
@@ -7878,7 +7883,7 @@
       </c>
       <c r="H43" s="3" t="inlineStr">
         <is>
-          <t>B_TYPE</t>
+          <t>EXT_B</t>
         </is>
       </c>
       <c r="I43" s="3" t="inlineStr">
@@ -7888,22 +7893,22 @@
       </c>
       <c r="J43" s="3" t="inlineStr">
         <is>
-          <t>SEL_RS2</t>
+          <t>ALU_B_RS2</t>
         </is>
       </c>
       <c r="K43" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>RAM_EXT_N</t>
         </is>
       </c>
       <c r="L43" s="3" t="inlineStr">
         <is>
-          <t>SEL_RS1</t>
+          <t>ALU_A_RS1</t>
         </is>
       </c>
       <c r="M43" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>RAM_WE_N</t>
         </is>
       </c>
       <c r="N43" s="3" t="inlineStr">
@@ -7941,7 +7946,7 @@
       </c>
       <c r="E44" s="3" t="inlineStr">
         <is>
-          <t>PC4</t>
+          <t>NPC_PC4</t>
         </is>
       </c>
       <c r="F44" s="3" t="inlineStr">
@@ -7956,7 +7961,7 @@
       </c>
       <c r="H44" s="3" t="inlineStr">
         <is>
-          <t>U_TYPE</t>
+          <t>EXT_U</t>
         </is>
       </c>
       <c r="I44" s="3" t="inlineStr">
@@ -7971,7 +7976,7 @@
       </c>
       <c r="K44" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>RAM_EXT_N</t>
         </is>
       </c>
       <c r="L44" s="3" t="inlineStr">
@@ -7981,7 +7986,7 @@
       </c>
       <c r="M44" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>RAM_WE_N</t>
         </is>
       </c>
       <c r="N44" s="3" t="inlineStr">
@@ -8019,7 +8024,7 @@
       </c>
       <c r="E45" s="3" t="inlineStr">
         <is>
-          <t>PC4</t>
+          <t>NPC_PC4</t>
         </is>
       </c>
       <c r="F45" s="3" t="inlineStr">
@@ -8034,7 +8039,7 @@
       </c>
       <c r="H45" s="3" t="inlineStr">
         <is>
-          <t>U_TYPE</t>
+          <t>EXT_U</t>
         </is>
       </c>
       <c r="I45" s="3" t="inlineStr">
@@ -8044,22 +8049,22 @@
       </c>
       <c r="J45" s="3" t="inlineStr">
         <is>
-          <t>SEL_EXT</t>
+          <t>ALU_B_EXT</t>
         </is>
       </c>
       <c r="K45" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>RAM_EXT_N</t>
         </is>
       </c>
       <c r="L45" s="3" t="inlineStr">
         <is>
-          <t>SEL_PC</t>
+          <t>ALU_A_PC</t>
         </is>
       </c>
       <c r="M45" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>RAM_WE_N</t>
         </is>
       </c>
       <c r="N45" s="3" t="inlineStr">
@@ -8097,7 +8102,7 @@
       </c>
       <c r="E46" s="3" t="inlineStr">
         <is>
-          <t>JUMP</t>
+          <t>NPC_JAL</t>
         </is>
       </c>
       <c r="F46" s="3" t="inlineStr">
@@ -8112,7 +8117,7 @@
       </c>
       <c r="H46" s="3" t="inlineStr">
         <is>
-          <t>J_TYPE</t>
+          <t>EXT_J</t>
         </is>
       </c>
       <c r="I46" s="3" t="inlineStr">
@@ -8127,7 +8132,7 @@
       </c>
       <c r="K46" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>RAM_EXT_N</t>
         </is>
       </c>
       <c r="L46" s="3" t="inlineStr">
@@ -8137,7 +8142,7 @@
       </c>
       <c r="M46" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>RAM_WE_N</t>
         </is>
       </c>
       <c r="N46" s="3" t="inlineStr">
@@ -8175,7 +8180,7 @@
       </c>
       <c r="E47" s="3" t="inlineStr">
         <is>
-          <t>JUMP</t>
+          <t>NPC_JALR</t>
         </is>
       </c>
       <c r="F47" s="3" t="inlineStr">
@@ -8190,7 +8195,7 @@
       </c>
       <c r="H47" s="3" t="inlineStr">
         <is>
-          <t>I_TYPE</t>
+          <t>EXT_I</t>
         </is>
       </c>
       <c r="I47" s="3" t="inlineStr">
@@ -8200,22 +8205,22 @@
       </c>
       <c r="J47" s="3" t="inlineStr">
         <is>
-          <t>SEL_EXT</t>
+          <t>ALU_B_EXT</t>
         </is>
       </c>
       <c r="K47" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>RAM_EXT_N</t>
         </is>
       </c>
       <c r="L47" s="3" t="inlineStr">
         <is>
-          <t>SEL_RS1</t>
+          <t>ALU_A_RS1</t>
         </is>
       </c>
       <c r="M47" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>RAM_WE_N</t>
         </is>
       </c>
       <c r="N47" s="3" t="inlineStr">
@@ -8263,7 +8268,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E55"/>
+  <dimension ref="A1:E57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -8335,8 +8340,8 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="n"/>
-      <c r="B4" s="3" t="n"/>
+      <c r="A4" s="8" t="n"/>
+      <c r="B4" s="8" t="n"/>
       <c r="C4" s="3" t="inlineStr">
         <is>
           <t>NPC_BRA</t>
@@ -8354,11 +8359,11 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="n"/>
-      <c r="B5" s="3" t="n"/>
+      <c r="A5" s="9" t="n"/>
+      <c r="B5" s="9" t="n"/>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>NPC_JMP</t>
+          <t>NPC_JAL</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
@@ -8368,970 +8373,898 @@
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>npc=PC+offset</t>
+          <t>npc = PC + offset (jal)</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>RF</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>rf_we</t>
-        </is>
-      </c>
+      <c r="A6" s="10" t="n"/>
+      <c r="B6" s="10" t="n"/>
       <c r="C6" s="3" t="inlineStr">
         <is>
+          <t>NPC_JALR</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>2'b01</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>npc = {alu_c[31:1], 1b0} (jalr)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="n"/>
+      <c r="B7" s="9" t="n"/>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
           <t>1'b1</t>
-        </is>
-      </c>
-      <c r="D6" s="5" t="inlineStr"/>
-      <c r="E6" s="3" t="inlineStr">
-        <is>
-          <t>允许写</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="3" t="n"/>
-      <c r="B7" s="3" t="n"/>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>1'b0</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr"/>
       <c r="E7" s="3" t="inlineStr">
         <is>
+          <t>允许写</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="n"/>
+      <c r="B8" s="9" t="n"/>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>1'b0</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr"/>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
           <t>禁止写</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t>WB_MUX</t>
-        </is>
-      </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>rf_wsel</t>
-        </is>
-      </c>
-      <c r="C8" s="3" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="8" t="n"/>
+      <c r="B9" s="8" t="n"/>
+      <c r="C9" s="3" t="inlineStr">
         <is>
           <t>WB_ALU</t>
         </is>
       </c>
-      <c r="D8" s="5" t="inlineStr">
+      <c r="D9" s="5" t="inlineStr">
         <is>
           <t>2'b00</t>
         </is>
       </c>
-      <c r="E8" s="3" t="inlineStr">
+      <c r="E9" s="3" t="inlineStr">
         <is>
           <t>wD=ALU.C</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="3" t="n"/>
-      <c r="B9" s="3" t="n"/>
-      <c r="C9" s="3" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="8" t="n"/>
+      <c r="B10" s="8" t="n"/>
+      <c r="C10" s="3" t="inlineStr">
         <is>
           <t>WB_RAM</t>
         </is>
       </c>
-      <c r="D9" s="5" t="inlineStr">
+      <c r="D10" s="5" t="inlineStr">
         <is>
           <t>2'b01</t>
         </is>
       </c>
-      <c r="E9" s="3" t="inlineStr">
+      <c r="E10" s="3" t="inlineStr">
         <is>
           <t>wD=MEXT.ext</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="3" t="n"/>
-      <c r="B10" s="3" t="n"/>
-      <c r="C10" s="3" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="9" t="n"/>
+      <c r="B11" s="9" t="n"/>
+      <c r="C11" s="3" t="inlineStr">
         <is>
           <t>WB_PC4</t>
         </is>
       </c>
-      <c r="D10" s="5" t="inlineStr">
+      <c r="D11" s="5" t="inlineStr">
         <is>
           <t>2'b10</t>
         </is>
       </c>
-      <c r="E10" s="3" t="inlineStr">
+      <c r="E11" s="3" t="inlineStr">
         <is>
           <t>wD=NPC.pc4(jal/jalr)</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="3" t="n"/>
-      <c r="B11" s="3" t="n"/>
-      <c r="C11" s="3" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="9" t="n"/>
+      <c r="B12" s="9" t="n"/>
+      <c r="C12" s="3" t="inlineStr">
         <is>
           <t>WB_EXT</t>
         </is>
       </c>
-      <c r="D11" s="5" t="inlineStr">
+      <c r="D12" s="5" t="inlineStr">
         <is>
           <t>2'b11</t>
         </is>
       </c>
-      <c r="E11" s="3" t="inlineStr">
+      <c r="E12" s="3" t="inlineStr">
         <is>
           <t>wD=SEXT.ext(lui)</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>SEXT</t>
-        </is>
-      </c>
-      <c r="B12" s="3" t="inlineStr">
-        <is>
-          <t>sext_op</t>
-        </is>
-      </c>
-      <c r="C12" s="3" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="8" t="n"/>
+      <c r="B13" s="8" t="n"/>
+      <c r="C13" s="3" t="inlineStr">
         <is>
           <t>EXT_I</t>
         </is>
       </c>
-      <c r="D12" s="5" t="inlineStr">
+      <c r="D13" s="5" t="inlineStr">
         <is>
           <t>3'b000</t>
         </is>
       </c>
-      <c r="E12" s="3" t="inlineStr">
+      <c r="E13" s="3" t="inlineStr">
         <is>
           <t>I型</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="3" t="n"/>
-      <c r="B13" s="3" t="n"/>
-      <c r="C13" s="3" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="8" t="n"/>
+      <c r="B14" s="8" t="n"/>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>EXT_S</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>3'b001</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>S型: {{20{imm[31]}}, imm[31:25], imm[11:7]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="9" t="n"/>
+      <c r="B15" s="9" t="n"/>
+      <c r="C15" s="3" t="inlineStr">
         <is>
           <t>EXT_B</t>
         </is>
       </c>
-      <c r="D13" s="5" t="inlineStr">
+      <c r="D15" s="5" t="inlineStr">
         <is>
           <t>3'b010</t>
         </is>
       </c>
-      <c r="E13" s="3" t="inlineStr">
+      <c r="E15" s="3" t="inlineStr">
         <is>
           <t>B型</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="3" t="n"/>
-      <c r="B14" s="3" t="n"/>
-      <c r="C14" s="3" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="9" t="n"/>
+      <c r="B16" s="9" t="n"/>
+      <c r="C16" s="3" t="inlineStr">
         <is>
           <t>EXT_U</t>
         </is>
       </c>
-      <c r="D14" s="5" t="inlineStr">
+      <c r="D16" s="5" t="inlineStr">
         <is>
           <t>3'b011</t>
         </is>
       </c>
-      <c r="E14" s="3" t="inlineStr">
+      <c r="E16" s="3" t="inlineStr">
         <is>
           <t>U型</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="3" t="n"/>
-      <c r="B15" s="3" t="n"/>
-      <c r="C15" s="3" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="8" t="n"/>
+      <c r="B17" s="8" t="n"/>
+      <c r="C17" s="3" t="inlineStr">
         <is>
           <t>EXT_J</t>
         </is>
       </c>
-      <c r="D15" s="5" t="inlineStr">
+      <c r="D17" s="5" t="inlineStr">
         <is>
           <t>3'b100</t>
         </is>
       </c>
-      <c r="E15" s="3" t="inlineStr">
+      <c r="E17" s="3" t="inlineStr">
         <is>
           <t>J型</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="3" t="inlineStr">
-        <is>
-          <t>ALU</t>
-        </is>
-      </c>
-      <c r="B16" s="3" t="inlineStr">
-        <is>
-          <t>alu_op</t>
-        </is>
-      </c>
-      <c r="C16" s="3" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="8" t="n"/>
+      <c r="B18" s="8" t="n"/>
+      <c r="C18" s="3" t="inlineStr">
         <is>
           <t>ALU_ADD</t>
         </is>
       </c>
-      <c r="D16" s="5" t="inlineStr">
+      <c r="D18" s="5" t="inlineStr">
         <is>
           <t>5'h00</t>
         </is>
       </c>
-      <c r="E16" s="3" t="inlineStr">
+      <c r="E18" s="3" t="inlineStr">
         <is>
           <t>C=A+B</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="3" t="n"/>
-      <c r="B17" s="3" t="n"/>
-      <c r="C17" s="3" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="8" t="n"/>
+      <c r="B19" s="8" t="n"/>
+      <c r="C19" s="3" t="inlineStr">
         <is>
           <t>ALU_SUB</t>
         </is>
       </c>
-      <c r="D17" s="5" t="inlineStr">
+      <c r="D19" s="5" t="inlineStr">
         <is>
           <t>5'h01</t>
         </is>
       </c>
-      <c r="E17" s="3" t="inlineStr">
+      <c r="E19" s="3" t="inlineStr">
         <is>
           <t>C=A-B</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="3" t="n"/>
-      <c r="B18" s="3" t="n"/>
-      <c r="C18" s="3" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="8" t="n"/>
+      <c r="B20" s="8" t="n"/>
+      <c r="C20" s="3" t="inlineStr">
         <is>
           <t>ALU_XOR</t>
         </is>
       </c>
-      <c r="D18" s="5" t="inlineStr">
+      <c r="D20" s="5" t="inlineStr">
         <is>
           <t>5'h02</t>
         </is>
       </c>
-      <c r="E18" s="3" t="inlineStr">
+      <c r="E20" s="3" t="inlineStr">
         <is>
           <t>C=A^B</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="3" t="n"/>
-      <c r="B19" s="3" t="n"/>
-      <c r="C19" s="3" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="8" t="n"/>
+      <c r="B21" s="8" t="n"/>
+      <c r="C21" s="3" t="inlineStr">
         <is>
           <t>ALU_OR</t>
         </is>
       </c>
-      <c r="D19" s="5" t="inlineStr">
+      <c r="D21" s="5" t="inlineStr">
         <is>
           <t>5'h03</t>
         </is>
       </c>
-      <c r="E19" s="3" t="inlineStr">
+      <c r="E21" s="3" t="inlineStr">
         <is>
           <t>C=A|B</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="3" t="n"/>
-      <c r="B20" s="3" t="n"/>
-      <c r="C20" s="3" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="8" t="n"/>
+      <c r="B22" s="8" t="n"/>
+      <c r="C22" s="3" t="inlineStr">
         <is>
           <t>ALU_AND</t>
         </is>
       </c>
-      <c r="D20" s="5" t="inlineStr">
+      <c r="D22" s="5" t="inlineStr">
         <is>
           <t>5'h04</t>
         </is>
       </c>
-      <c r="E20" s="3" t="inlineStr">
+      <c r="E22" s="3" t="inlineStr">
         <is>
           <t>C=A&amp;B</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="3" t="n"/>
-      <c r="B21" s="3" t="n"/>
-      <c r="C21" s="3" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="8" t="n"/>
+      <c r="B23" s="8" t="n"/>
+      <c r="C23" s="3" t="inlineStr">
         <is>
           <t>ALU_SLL</t>
         </is>
       </c>
-      <c r="D21" s="5" t="inlineStr">
+      <c r="D23" s="5" t="inlineStr">
         <is>
           <t>5'h05</t>
         </is>
       </c>
-      <c r="E21" s="3" t="inlineStr">
-        <is>
-          <t>C=A&lt;&lt;B</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="3" t="n"/>
-      <c r="B22" s="3" t="n"/>
-      <c r="C22" s="3" t="inlineStr">
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>C=A&lt;&lt;B[4:0]</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="8" t="n"/>
+      <c r="B24" s="8" t="n"/>
+      <c r="C24" s="3" t="inlineStr">
         <is>
           <t>ALU_SRL</t>
         </is>
       </c>
-      <c r="D22" s="5" t="inlineStr">
+      <c r="D24" s="5" t="inlineStr">
         <is>
           <t>5'h06</t>
         </is>
       </c>
-      <c r="E22" s="3" t="inlineStr">
-        <is>
-          <t>C=A&gt;&gt;B</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="3" t="n"/>
-      <c r="B23" s="3" t="n"/>
-      <c r="C23" s="3" t="inlineStr">
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>C=A&gt;&gt;B[4:0](逻辑)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="8" t="n"/>
+      <c r="B25" s="8" t="n"/>
+      <c r="C25" s="3" t="inlineStr">
         <is>
           <t>ALU_SRA</t>
         </is>
       </c>
-      <c r="D23" s="5" t="inlineStr">
+      <c r="D25" s="5" t="inlineStr">
         <is>
           <t>5'h07</t>
         </is>
       </c>
-      <c r="E23" s="3" t="inlineStr">
-        <is>
-          <t>C=A&gt;&gt;&gt;B</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="3" t="n"/>
-      <c r="B24" s="3" t="n"/>
-      <c r="C24" s="3" t="inlineStr">
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>C=$signed(A)&gt;&gt;&gt;B[4:0](算术)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="8" t="n"/>
+      <c r="B26" s="8" t="n"/>
+      <c r="C26" s="3" t="inlineStr">
         <is>
           <t>ALU_EQ</t>
         </is>
       </c>
-      <c r="D24" s="5" t="inlineStr">
+      <c r="D26" s="5" t="inlineStr">
         <is>
           <t>5'h08</t>
         </is>
       </c>
-      <c r="E24" s="3" t="inlineStr">
+      <c r="E26" s="3" t="inlineStr">
         <is>
           <t>br=(A==B)</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="3" t="n"/>
-      <c r="B25" s="3" t="n"/>
-      <c r="C25" s="3" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="8" t="n"/>
+      <c r="B27" s="8" t="n"/>
+      <c r="C27" s="3" t="inlineStr">
         <is>
           <t>ALU_NE</t>
         </is>
       </c>
-      <c r="D25" s="5" t="inlineStr">
+      <c r="D27" s="5" t="inlineStr">
         <is>
           <t>5'h09</t>
         </is>
       </c>
-      <c r="E25" s="3" t="inlineStr">
+      <c r="E27" s="3" t="inlineStr">
         <is>
           <t>br=(A!=B)</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="3" t="n"/>
-      <c r="B26" s="3" t="n"/>
-      <c r="C26" s="3" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="8" t="n"/>
+      <c r="B28" s="8" t="n"/>
+      <c r="C28" s="3" t="inlineStr">
         <is>
           <t>ALU_SLT</t>
         </is>
       </c>
-      <c r="D26" s="5" t="inlineStr">
+      <c r="D28" s="5" t="inlineStr">
         <is>
           <t>5'h0A</t>
         </is>
       </c>
-      <c r="E26" s="3" t="inlineStr">
+      <c r="E28" s="3" t="inlineStr">
         <is>
           <t>br/C=(A&lt;B)</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="3" t="n"/>
-      <c r="B27" s="3" t="n"/>
-      <c r="C27" s="3" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="8" t="n"/>
+      <c r="B29" s="8" t="n"/>
+      <c r="C29" s="3" t="inlineStr">
         <is>
           <t>ALU_SLTU</t>
         </is>
       </c>
-      <c r="D27" s="5" t="inlineStr">
+      <c r="D29" s="5" t="inlineStr">
         <is>
           <t>5'h0B</t>
         </is>
       </c>
-      <c r="E27" s="3" t="inlineStr">
+      <c r="E29" s="3" t="inlineStr">
         <is>
           <t>br/C=(A&lt;B)U</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="3" t="n"/>
-      <c r="B28" s="3" t="n"/>
-      <c r="C28" s="3" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="8" t="n"/>
+      <c r="B30" s="8" t="n"/>
+      <c r="C30" s="3" t="inlineStr">
         <is>
           <t>ALU_MUL</t>
         </is>
       </c>
-      <c r="D28" s="5" t="inlineStr">
+      <c r="D30" s="5" t="inlineStr">
         <is>
           <t>5'h10</t>
         </is>
       </c>
-      <c r="E28" s="3" t="inlineStr">
+      <c r="E30" s="3" t="inlineStr">
         <is>
           <t>C=(A×B)[31:0]</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="3" t="n"/>
-      <c r="B29" s="3" t="n"/>
-      <c r="C29" s="3" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="8" t="n"/>
+      <c r="B31" s="8" t="n"/>
+      <c r="C31" s="3" t="inlineStr">
         <is>
           <t>ALU_MULH</t>
         </is>
       </c>
-      <c r="D29" s="5" t="inlineStr">
+      <c r="D31" s="5" t="inlineStr">
         <is>
           <t>5'h11</t>
         </is>
       </c>
-      <c r="E29" s="3" t="inlineStr">
+      <c r="E31" s="3" t="inlineStr">
         <is>
           <t>C=(A×B)[63:32]</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="3" t="n"/>
-      <c r="B30" s="3" t="n"/>
-      <c r="C30" s="3" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="8" t="n"/>
+      <c r="B32" s="8" t="n"/>
+      <c r="C32" s="3" t="inlineStr">
         <is>
           <t>ALU_MULHU</t>
         </is>
       </c>
-      <c r="D30" s="5" t="inlineStr">
+      <c r="D32" s="5" t="inlineStr">
         <is>
           <t>5'h12</t>
         </is>
       </c>
-      <c r="E30" s="3" t="inlineStr">
+      <c r="E32" s="3" t="inlineStr">
         <is>
           <t>C=(A×B)[63:32]U</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="3" t="n"/>
-      <c r="B31" s="3" t="n"/>
-      <c r="C31" s="3" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="8" t="n"/>
+      <c r="B33" s="8" t="n"/>
+      <c r="C33" s="3" t="inlineStr">
         <is>
           <t>ALU_DIV</t>
         </is>
       </c>
-      <c r="D31" s="5" t="inlineStr">
+      <c r="D33" s="5" t="inlineStr">
         <is>
           <t>5'h13</t>
         </is>
       </c>
-      <c r="E31" s="3" t="inlineStr">
+      <c r="E33" s="3" t="inlineStr">
         <is>
           <t>C=A/B</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="3" t="n"/>
-      <c r="B32" s="3" t="n"/>
-      <c r="C32" s="3" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="8" t="n"/>
+      <c r="B34" s="8" t="n"/>
+      <c r="C34" s="3" t="inlineStr">
         <is>
           <t>ALU_DIVU</t>
         </is>
       </c>
-      <c r="D32" s="5" t="inlineStr">
+      <c r="D34" s="5" t="inlineStr">
         <is>
           <t>5'h14</t>
         </is>
       </c>
-      <c r="E32" s="3" t="inlineStr">
+      <c r="E34" s="3" t="inlineStr">
         <is>
           <t>C=A/B U</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="3" t="n"/>
-      <c r="B33" s="3" t="n"/>
-      <c r="C33" s="3" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="8" t="n"/>
+      <c r="B35" s="8" t="n"/>
+      <c r="C35" s="3" t="inlineStr">
         <is>
           <t>ALU_REM</t>
         </is>
       </c>
-      <c r="D33" s="5" t="inlineStr">
+      <c r="D35" s="5" t="inlineStr">
         <is>
           <t>5'h15</t>
         </is>
       </c>
-      <c r="E33" s="3" t="inlineStr">
+      <c r="E35" s="3" t="inlineStr">
         <is>
           <t>C=A%B</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="3" t="n"/>
-      <c r="B34" s="3" t="n"/>
-      <c r="C34" s="3" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="9" t="n"/>
+      <c r="B36" s="9" t="n"/>
+      <c r="C36" s="3" t="inlineStr">
         <is>
           <t>ALU_REMU</t>
         </is>
       </c>
-      <c r="D34" s="5" t="inlineStr">
+      <c r="D36" s="5" t="inlineStr">
         <is>
           <t>5'h16</t>
         </is>
       </c>
-      <c r="E34" s="3" t="inlineStr">
+      <c r="E36" s="3" t="inlineStr">
         <is>
           <t>C=A%B U</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="3" t="n"/>
-      <c r="B35" s="3" t="n"/>
-      <c r="C35" s="3" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="9" t="n"/>
+      <c r="B37" s="9" t="n"/>
+      <c r="C37" s="3" t="inlineStr">
         <is>
           <t>ALU_GE</t>
         </is>
       </c>
-      <c r="D35" s="5" t="inlineStr">
+      <c r="D37" s="5" t="inlineStr">
         <is>
           <t>5'h17</t>
         </is>
       </c>
-      <c r="E35" s="3" t="inlineStr">
+      <c r="E37" s="3" t="inlineStr">
         <is>
           <t>br=(A&gt;=B)</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="3" t="n"/>
-      <c r="B36" s="3" t="n"/>
-      <c r="C36" s="3" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="9" t="n"/>
+      <c r="B38" s="9" t="n"/>
+      <c r="C38" s="3" t="inlineStr">
         <is>
           <t>ALU_GEU</t>
         </is>
       </c>
-      <c r="D36" s="5" t="inlineStr">
+      <c r="D38" s="5" t="inlineStr">
         <is>
           <t>5'h18</t>
         </is>
       </c>
-      <c r="E36" s="3" t="inlineStr">
+      <c r="E38" s="3" t="inlineStr">
         <is>
           <t>br=(A&gt;=B)U</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="3" t="inlineStr">
-        <is>
-          <t>ALU(A MUX)</t>
-        </is>
-      </c>
-      <c r="B37" s="3" t="inlineStr">
-        <is>
-          <t>alua_sel</t>
-        </is>
-      </c>
-      <c r="C37" s="3" t="inlineStr">
+    <row r="39">
+      <c r="A39" s="9" t="n"/>
+      <c r="B39" s="9" t="n"/>
+      <c r="C39" s="3" t="inlineStr">
         <is>
           <t>ALU_A_RS1</t>
         </is>
       </c>
-      <c r="D37" s="5" t="inlineStr">
+      <c r="D39" s="5" t="inlineStr">
         <is>
           <t>1'b0</t>
         </is>
       </c>
-      <c r="E37" s="3" t="inlineStr">
+      <c r="E39" s="3" t="inlineStr">
         <is>
           <t>A=RF.rD1</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="3" t="n"/>
-      <c r="B38" s="3" t="n"/>
-      <c r="C38" s="3" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="9" t="n"/>
+      <c r="B40" s="9" t="n"/>
+      <c r="C40" s="3" t="inlineStr">
         <is>
           <t>ALU_A_PC</t>
         </is>
       </c>
-      <c r="D38" s="5" t="inlineStr">
+      <c r="D40" s="5" t="inlineStr">
         <is>
           <t>1'b1</t>
         </is>
       </c>
-      <c r="E38" s="3" t="inlineStr">
+      <c r="E40" s="3" t="inlineStr">
         <is>
           <t>A=PC(auipc)</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="3" t="inlineStr">
-        <is>
-          <t>ALU(B MUX)</t>
-        </is>
-      </c>
-      <c r="B39" s="3" t="inlineStr">
-        <is>
-          <t>alub_sel</t>
-        </is>
-      </c>
-      <c r="C39" s="3" t="inlineStr">
+    <row r="41">
+      <c r="A41" s="9" t="n"/>
+      <c r="B41" s="9" t="n"/>
+      <c r="C41" s="3" t="inlineStr">
         <is>
           <t>ALU_B_RS2</t>
         </is>
       </c>
-      <c r="D39" s="5" t="inlineStr">
+      <c r="D41" s="5" t="inlineStr">
         <is>
           <t>1'b0</t>
         </is>
       </c>
-      <c r="E39" s="3" t="inlineStr">
+      <c r="E41" s="3" t="inlineStr">
         <is>
           <t>B=RF.rD2</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="3" t="n"/>
-      <c r="B40" s="3" t="n"/>
-      <c r="C40" s="3" t="inlineStr">
+    <row r="42">
+      <c r="A42" s="8" t="n"/>
+      <c r="B42" s="8" t="n"/>
+      <c r="C42" s="3" t="inlineStr">
         <is>
           <t>ALU_B_EXT</t>
         </is>
       </c>
-      <c r="D40" s="5" t="inlineStr">
+      <c r="D42" s="5" t="inlineStr">
         <is>
           <t>1'b1</t>
         </is>
       </c>
-      <c r="E40" s="3" t="inlineStr">
+      <c r="E42" s="3" t="inlineStr">
         <is>
           <t>B=SEXT.ext</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="3" t="inlineStr">
-        <is>
-          <t>MREQ,MEXT</t>
-        </is>
-      </c>
-      <c r="B41" s="3" t="inlineStr">
-        <is>
-          <t>ram_rop</t>
-        </is>
-      </c>
-      <c r="C41" s="3" t="inlineStr">
+    <row r="43">
+      <c r="A43" s="8" t="n"/>
+      <c r="B43" s="8" t="n"/>
+      <c r="C43" s="3" t="inlineStr">
         <is>
           <t>RAM_EXT_N</t>
         </is>
       </c>
-      <c r="D41" s="5" t="inlineStr">
+      <c r="D43" s="5" t="inlineStr">
         <is>
           <t>3'b000</t>
         </is>
       </c>
-      <c r="E41" s="3" t="inlineStr">
+      <c r="E43" s="3" t="inlineStr">
         <is>
           <t>不读</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="3" t="n"/>
-      <c r="B42" s="3" t="n"/>
-      <c r="C42" s="3" t="inlineStr">
+    <row r="44">
+      <c r="A44" s="8" t="n"/>
+      <c r="B44" s="8" t="n"/>
+      <c r="C44" s="3" t="inlineStr">
         <is>
           <t>RAM_EXT_B</t>
         </is>
       </c>
-      <c r="D42" s="5" t="inlineStr">
+      <c r="D44" s="5" t="inlineStr">
         <is>
           <t>3'b001</t>
         </is>
       </c>
-      <c r="E42" s="3" t="inlineStr">
+      <c r="E44" s="3" t="inlineStr">
         <is>
           <t>lb</t>
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="3" t="n"/>
-      <c r="B43" s="3" t="n"/>
-      <c r="C43" s="3" t="inlineStr">
+    <row r="45">
+      <c r="A45" s="8" t="n"/>
+      <c r="B45" s="8" t="n"/>
+      <c r="C45" s="3" t="inlineStr">
         <is>
           <t>RAM_EXT_BU</t>
         </is>
       </c>
-      <c r="D43" s="5" t="inlineStr">
+      <c r="D45" s="5" t="inlineStr">
         <is>
           <t>3'b011</t>
         </is>
       </c>
-      <c r="E43" s="3" t="inlineStr">
+      <c r="E45" s="3" t="inlineStr">
         <is>
           <t>lbu</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="3" t="n"/>
-      <c r="B44" s="3" t="n"/>
-      <c r="C44" s="3" t="inlineStr">
+    <row r="46">
+      <c r="A46" s="9" t="n"/>
+      <c r="B46" s="9" t="n"/>
+      <c r="C46" s="3" t="inlineStr">
         <is>
           <t>RAM_EXT_H</t>
         </is>
       </c>
-      <c r="D44" s="5" t="inlineStr">
+      <c r="D46" s="5" t="inlineStr">
         <is>
           <t>3'b100</t>
         </is>
       </c>
-      <c r="E44" s="3" t="inlineStr">
+      <c r="E46" s="3" t="inlineStr">
         <is>
           <t>lh</t>
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" s="3" t="n"/>
-      <c r="B45" s="3" t="n"/>
-      <c r="C45" s="3" t="inlineStr">
+    <row r="47">
+      <c r="A47" s="9" t="n"/>
+      <c r="B47" s="9" t="n"/>
+      <c r="C47" s="3" t="inlineStr">
         <is>
           <t>RAM_EXT_HU</t>
         </is>
       </c>
-      <c r="D45" s="5" t="inlineStr">
+      <c r="D47" s="5" t="inlineStr">
         <is>
           <t>3'b101</t>
         </is>
       </c>
-      <c r="E45" s="3" t="inlineStr">
+      <c r="E47" s="3" t="inlineStr">
         <is>
           <t>lhu</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" s="3" t="n"/>
-      <c r="B46" s="3" t="n"/>
-      <c r="C46" s="3" t="inlineStr">
+    <row r="48">
+      <c r="A48" s="8" t="n"/>
+      <c r="B48" s="8" t="n"/>
+      <c r="C48" s="3" t="inlineStr">
         <is>
           <t>RAM_EXT_W</t>
         </is>
       </c>
-      <c r="D46" s="5" t="inlineStr">
+      <c r="D48" s="5" t="inlineStr">
         <is>
           <t>3'b010</t>
         </is>
       </c>
-      <c r="E46" s="3" t="inlineStr">
+      <c r="E48" s="3" t="inlineStr">
         <is>
           <t>lw</t>
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" s="3" t="inlineStr">
-        <is>
-          <t>MREQ</t>
-        </is>
-      </c>
-      <c r="B47" s="3" t="inlineStr">
-        <is>
-          <t>ram_wop</t>
-        </is>
-      </c>
-      <c r="C47" s="3" t="inlineStr">
+    <row r="49">
+      <c r="A49" s="8" t="n"/>
+      <c r="B49" s="8" t="n"/>
+      <c r="C49" s="3" t="inlineStr">
         <is>
           <t>RAM_WE_N</t>
         </is>
       </c>
-      <c r="D47" s="5" t="inlineStr">
+      <c r="D49" s="5" t="inlineStr">
         <is>
           <t>4'b0000</t>
         </is>
       </c>
-      <c r="E47" s="3" t="inlineStr">
+      <c r="E49" s="3" t="inlineStr">
         <is>
           <t>不写</t>
         </is>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" s="3" t="n"/>
-      <c r="B48" s="3" t="n"/>
-      <c r="C48" s="3" t="inlineStr">
+    <row r="50">
+      <c r="A50" s="9" t="n"/>
+      <c r="B50" s="9" t="n"/>
+      <c r="C50" s="3" t="inlineStr">
         <is>
           <t>RAM_WE_B</t>
         </is>
       </c>
-      <c r="D48" s="5" t="inlineStr">
+      <c r="D50" s="5" t="inlineStr">
         <is>
           <t>4'b0001</t>
         </is>
       </c>
-      <c r="E48" s="3" t="inlineStr">
+      <c r="E50" s="3" t="inlineStr">
         <is>
           <t>sb</t>
         </is>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" s="3" t="n"/>
-      <c r="B49" s="3" t="n"/>
-      <c r="C49" s="3" t="inlineStr">
+    <row r="51">
+      <c r="A51" s="9" t="n"/>
+      <c r="B51" s="9" t="n"/>
+      <c r="C51" s="3" t="inlineStr">
         <is>
           <t>RAM_WE_H</t>
         </is>
       </c>
-      <c r="D49" s="5" t="inlineStr">
+      <c r="D51" s="5" t="inlineStr">
         <is>
           <t>4'b0011</t>
         </is>
       </c>
-      <c r="E49" s="3" t="inlineStr">
+      <c r="E51" s="3" t="inlineStr">
         <is>
           <t>sh</t>
         </is>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" s="3" t="n"/>
-      <c r="B50" s="3" t="n"/>
-      <c r="C50" s="3" t="inlineStr">
+    <row r="52">
+      <c r="A52" s="9" t="n"/>
+      <c r="B52" s="9" t="n"/>
+      <c r="C52" s="3" t="inlineStr">
         <is>
           <t>RAM_WE_W</t>
         </is>
       </c>
-      <c r="D50" s="5" t="inlineStr">
+      <c r="D52" s="5" t="inlineStr">
         <is>
           <t>4'b1111</t>
         </is>
       </c>
-      <c r="E50" s="3" t="inlineStr">
+      <c r="E52" s="3" t="inlineStr">
         <is>
           <t>sw</t>
         </is>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" s="3" t="inlineStr">
-        <is>
-          <t>ALU(core)</t>
-        </is>
-      </c>
-      <c r="B51" s="3" t="inlineStr">
-        <is>
-          <t>is_mul</t>
-        </is>
-      </c>
-      <c r="C51" s="3" t="inlineStr">
-        <is>
-          <t>1'b1</t>
-        </is>
-      </c>
-      <c r="D51" s="5" t="inlineStr"/>
-      <c r="E51" s="3" t="inlineStr">
-        <is>
-          <t>乘法stall</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="3" t="n"/>
-      <c r="B52" s="3" t="n"/>
-      <c r="C52" s="3" t="inlineStr">
-        <is>
-          <t>1'b0</t>
-        </is>
-      </c>
-      <c r="D52" s="5" t="inlineStr"/>
-      <c r="E52" s="3" t="inlineStr">
-        <is>
-          <t>非乘法</t>
-        </is>
-      </c>
-    </row>
     <row r="53">
-      <c r="A53" s="3" t="inlineStr">
-        <is>
-          <t>ALU(core)</t>
-        </is>
-      </c>
-      <c r="B53" s="3" t="inlineStr">
-        <is>
-          <t>is_div</t>
-        </is>
-      </c>
+      <c r="A53" s="9" t="n"/>
+      <c r="B53" s="9" t="n"/>
       <c r="C53" s="3" t="inlineStr">
         <is>
           <t>1'b1</t>
@@ -9340,13 +9273,13 @@
       <c r="D53" s="5" t="inlineStr"/>
       <c r="E53" s="3" t="inlineStr">
         <is>
-          <t>除法stall</t>
+          <t>乘法stall</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="3" t="n"/>
-      <c r="B54" s="3" t="n"/>
+      <c r="A54" s="9" t="n"/>
+      <c r="B54" s="9" t="n"/>
       <c r="C54" s="3" t="inlineStr">
         <is>
           <t>1'b0</t>
@@ -9355,28 +9288,58 @@
       <c r="D54" s="5" t="inlineStr"/>
       <c r="E54" s="3" t="inlineStr">
         <is>
+          <t>非乘法</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="9" t="n"/>
+      <c r="B55" s="9" t="n"/>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>1'b1</t>
+        </is>
+      </c>
+      <c r="D55" s="5" t="inlineStr"/>
+      <c r="E55" s="3" t="inlineStr">
+        <is>
+          <t>除法stall</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="9" t="n"/>
+      <c r="B56" s="9" t="n"/>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>1'b0</t>
+        </is>
+      </c>
+      <c r="D56" s="5" t="inlineStr"/>
+      <c r="E56" s="3" t="inlineStr">
+        <is>
           <t>非除法</t>
         </is>
       </c>
     </row>
-    <row r="55">
-      <c r="A55" s="3" t="inlineStr">
+    <row r="57">
+      <c r="A57" s="3" t="inlineStr">
         <is>
           <t>PC</t>
         </is>
       </c>
-      <c r="B55" s="3" t="inlineStr"/>
-      <c r="C55" s="3" t="inlineStr">
+      <c r="B57" s="3" t="inlineStr"/>
+      <c r="C57" s="3" t="inlineStr">
         <is>
           <t>PC_INIT_VAL</t>
         </is>
       </c>
-      <c r="D55" s="5" t="inlineStr">
+      <c r="D57" s="5" t="inlineStr">
         <is>
           <t>32'h0</t>
         </is>
       </c>
-      <c r="E55" s="3" t="inlineStr">
+      <c r="E57" s="3" t="inlineStr">
         <is>
           <t>PC初值</t>
         </is>

</xml_diff>